<commit_message>
added desc of genesis
</commit_message>
<xml_diff>
--- a/public/data/upcoming-events.xlsx
+++ b/public/data/upcoming-events.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Event name</t>
   </si>
@@ -443,7 +443,9 @@
       <c r="B2" s="1"/>
       <c r="C2" s="3"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="F2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">

</xml_diff>